<commit_message>
write script for Idp Search
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/IdpData.xlsx
+++ b/src/test/resources/testdata/IdpData.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Gyrus_Selenium_Automation\GyrusAim17_Learner_Automation\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DED3FEB0-C482-46D5-9153-AD2F0F751E04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E521B85-0865-437F-B769-CBFEF791F809}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{B7C73089-E2C0-4EF9-A86E-1C7B29356A86}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{B7C73089-E2C0-4EF9-A86E-1C7B29356A86}"/>
   </bookViews>
   <sheets>
     <sheet name="FilterRating" sheetId="1" r:id="rId1"/>
     <sheet name="FilterDueDate" sheetId="2" r:id="rId2"/>
+    <sheet name="SearchData" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Rating</t>
   </si>
@@ -49,6 +50,24 @@
   </si>
   <si>
     <t>Overdue</t>
+  </si>
+  <si>
+    <t>TEST01 Document by org -SU1-T354</t>
+  </si>
+  <si>
+    <t>SearchValid</t>
+  </si>
+  <si>
+    <t>SearchInValid</t>
+  </si>
+  <si>
+    <t>jhjghfjhgjfhgj</t>
+  </si>
+  <si>
+    <t>SearchPartial</t>
+  </si>
+  <si>
+    <t>Test</t>
   </si>
 </sst>
 </file>
@@ -474,4 +493,41 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD1911BD-E014-4C06-9120-3EA868E0774C}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="29.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="12.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>